<commit_message>
Save library recording Session 14/10/2026, 01:45:44 - 24723b38-b0b6-4d75-a9b0-c425ca37fb0d - 2026-10-13T14:56:20.018779Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/24723b38-b0b6-4d75-a9b0-c425ca37fb0d/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/24723b38-b0b6-4d75-a9b0-c425ca37fb0d/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,948 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://www.harrisfarm.com.au/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.harrisfarm.com.au/</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click DELIVERY</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-find-flow &gt; div:nth-of-type(1) &gt; button:nth-of-type(3)", "x": 651, "y": 506, "text": "DELIVERY", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Click e.g. 2066</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-postcode", "x": 476, "y": 474, "text": "e.g. 2066", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Type: 2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-postcode"}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Type: 0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-postcode"}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>step-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Type: 4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-postcode"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>step-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Type: 7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-postcode"}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>step-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Click CHECK DELIVERY</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-find", "x": 659, "y": 464, "text": "CHECK DELIVERY", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>step-008.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Click CONTINUE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-select-slot", "x": 413, "y": 542, "text": "CONTINUE", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>step-009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Click THU
+15 Oct</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-days &gt; button:nth-of-type(2)", "x": 474, "y": 168, "text": "THU\n15 Oct", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>step-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Click Afternoon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-periods &gt; button:nth-of-type(2)", "x": 528, "y": 260, "text": "Afternoon", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>step-011.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Click 12:00 PM-1:00 PM
+12:30 PM-1:30 PM
+1:00 PM-2:00 PM
+1:30 PM-2:30 PM
+2:00 PM-3:00 P</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-slots", "x": 617, "y": 409, "text": "12:00 PM-1:00 PM\n12:30 PM-1:30 PM\n1:00 PM-2:00 PM\n1:30 PM-2:30 PM\n2:00 PM-3:00 P", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>step-012.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Click 12:30 PM-1:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-slots &gt; button:nth-of-type(2)", "x": 591, "y": 390, "text": "12:30 PM-1:30 PM", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>step-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Click RESERVE TIME</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-reserve", "x": 633, "y": 584, "text": "RESERVE TIME", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>step-014.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Click Same day express delivery 🍉🥑</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"primary": "#shopify-section-sections--19725413744699__announcement-bar &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1)", "x": 405, "y": 29, "text": "Same day express delivery \ud83c\udf49\ud83e\udd51", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>step-015.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Click Search</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{"primary": "#Search-In-Template", "x": 390, "y": 61, "text": "Search", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>step-016.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Type: {{Product1}}</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>{{Product1}}</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{"primary": "#Search-In-Modal"}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>step-017.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Click ADD TO CART</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{"primary": "button[name=\"add\"]", "x": 411, "y": 464, "text": "ADD TO CART", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>step-018.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Click ADD TO CART</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{"primary": "button[name=\"add\"]", "x": 670, "y": 464, "text": "ADD TO CART", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>step-019.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Click ADD TO CART</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{"primary": "button[name=\"add\"]", "x": 892, "y": 495, "text": "ADD TO CART", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>step-020.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Click 413,451</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{"primary": "#predictive-search-option-product-1 &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; a:nth-of-type(1)", "x": 413, "y": 451, "text": "", "tag": "a"}</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Click 411,464</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>{"primary": null, "x": 411, "y": 464, "text": null, "tag": null}</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Click Apple Granny Smith Organic 1kg
+AUSTRALIA
+$12.99 EA $12.99 / kg
+ADD TO CART
+Apple</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{"primary": "#MainProduct-template--19725411582011__main &gt; div:nth-of-type(1) &gt; div:nth-of-type(2)", "x": 476, "y": 464, "text": "Apple Granny Smith Organic 1kg\nAUSTRALIA\n$12.99 EA $12.99 / kg\nADD TO CART\nApple", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>step-023.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Click Apple Granny Smith Organic</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>{"primary": "#ProductInfo-template--19725411582011__main &gt; div:nth-of-type(3) &gt; h3:nth-of-type(1)", "x": 712, "y": 458, "text": "Apple Granny Smith Organic", "tag": "h3"}</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>step-024.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Click Apple Granny Smith Organic
+Crisp and tangy, our Apple Granny Smith Organic 1kg</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{"primary": "#ProductInfo-template--19725411582011__main &gt; div:nth-of-type(3)", "x": 937, "y": 474, "text": "Apple Granny Smith Organic\n\nCrisp and tangy, our Apple Granny Smith Organic 1kg ", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>step-025.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Click ADD TO CART</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>{"primary": "#ProductInfo-template--19725411582011__main &gt; div:nth-of-type(2) &gt; div:nth-of-type(4)", "x": 678, "y": 338, "text": "ADD TO CART", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>step-026.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Click 675,370</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>{"primary": "#product-form-142501355 &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(2)", "x": 675, "y": 370, "text": "", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>step-027.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Click 709,351</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>{"primary": "#product-form-142501355 &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(2)", "x": 709, "y": 351, "text": "", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>step-028.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Click 701,349</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>{"primary": "#product-form-142501355 &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(2)", "x": 701, "y": 349, "text": "", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>step-029.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Click 696,354</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>{"primary": "#product-form-142501355 &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(2)", "x": 696, "y": 354, "text": "", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>step-030.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Click ADD TO CART</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>{"primary": "#ProductInfo-template--19725411582011__main &gt; div:nth-of-type(2) &gt; div:nth-of-type(4)", "x": 709, "y": 333, "text": "ADD TO CART", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>step-031.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Click $67.53</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-icon-bubble &gt; div:nth-of-type(1) &gt; span:nth-of-type(2)", "x": 957, "y": 63, "text": "$67.53", "tag": "span"}</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>step-032.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Session 14/10/2026, 01:45:44</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Click VIEW CART</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>{"primary": "button[aria-label=\"View cart\"]", "x": 829, "y": 589, "text": "VIEW CART", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Save library recording Session 14/10/2026, 01:45:44 - 24723b38-b0b6-4d75-a9b0-c425ca37fb0d - 2026-10-13T14:57:56.527489Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/24723b38-b0b6-4d75-a9b0-c425ca37fb0d/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/24723b38-b0b6-4d75-a9b0-c425ca37fb0d/resources/azure-devops.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>{{Order_Qty}}</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>{{store_picker_postcode}}</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>{{store_picker_postcode_2}}</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>{{store_picker_postcode_3}}</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>